<commit_message>
CRM import updates existing clients by CQC location ID; manager names for all priority providers; named first emails
Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_01XByJMQfkaq2do2XmLu4Dhj
</commit_message>
<xml_diff>
--- a/documents/Haverton Recruitment/8 First Client/This Week 20 Providers.xlsx
+++ b/documents/Haverton Recruitment/8 First Client/This Week 20 Providers.xlsx
@@ -24,7 +24,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="261" uniqueCount="199">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="281" uniqueCount="219">
   <si>
     <t xml:space="preserve">This Week: 20 Providers to Contact</t>
   </si>
@@ -122,6 +122,9 @@
     <t xml:space="preserve">Registered Manager vacancy advertised on Indeed (posted 18 Sep 2026, Tonbridge)</t>
   </si>
   <si>
+    <t xml:space="preserve">Miss Usebia Muzondo (Registered Manager)</t>
+  </si>
+  <si>
     <t xml:space="preserve">Radfield Home Care Bromley, Orpington &amp; Beckenham</t>
   </si>
   <si>
@@ -146,6 +149,9 @@
     <t xml:space="preserve">Care Assistant vacancy advertised on Indeed (posted 17 Sep 2026, Orpington)</t>
   </si>
   <si>
+    <t xml:space="preserve">Miss Chanice Cassandra Baugh-Fredericks (Registered Manager)</t>
+  </si>
+  <si>
     <t xml:space="preserve">Lauriem White Oak Court (EC)</t>
   </si>
   <si>
@@ -167,6 +173,9 @@
     <t xml:space="preserve">Care Assistant vacancy in Swanley advertised on Indeed (posted 23 Sep 2026)</t>
   </si>
   <si>
+    <t xml:space="preserve">Mrs Stephanie Christina Kimberley Hasleham (Registered Manager)</t>
+  </si>
+  <si>
     <t xml:space="preserve">Homesdale Supported Living</t>
   </si>
   <si>
@@ -194,6 +203,9 @@
     <t xml:space="preserve">Lead Support Worker vacancy advertised on Indeed (posted 24 Sep 2026, Chislehurst)</t>
   </si>
   <si>
+    <t xml:space="preserve">Mr Brett Anthony Rutter (Registered Manager)</t>
+  </si>
+  <si>
     <t xml:space="preserve">Home Instead</t>
   </si>
   <si>
@@ -215,6 +227,9 @@
     <t xml:space="preserve">Care Assistant vacancy in Dartford advertised on Indeed (posted 20 Aug 2026; check it is still open)</t>
   </si>
   <si>
+    <t xml:space="preserve">Mr Ram Chandra Thapa (Nominated Individual)</t>
+  </si>
+  <si>
     <t xml:space="preserve">B</t>
   </si>
   <si>
@@ -239,6 +254,9 @@
     <t xml:space="preserve">Nursing home 1.2 miles from Swanley</t>
   </si>
   <si>
+    <t xml:space="preserve">Mrs Damilola Abimbola Baiyewu (Registered Manager)</t>
+  </si>
+  <si>
     <t xml:space="preserve">Kentwood House</t>
   </si>
   <si>
@@ -260,6 +278,9 @@
     <t xml:space="preserve">Independent nursing home near Dartford</t>
   </si>
   <si>
+    <t xml:space="preserve">Mrs Sarika Puthalath (Registered Manager)</t>
+  </si>
+  <si>
     <t xml:space="preserve">West Hill Care Home</t>
   </si>
   <si>
@@ -284,6 +305,9 @@
     <t xml:space="preserve">Independent nursing home in Dartford with its own careers page</t>
   </si>
   <si>
+    <t xml:space="preserve">Miss Lauren Justine Griffin (Registered Manager)</t>
+  </si>
+  <si>
     <t xml:space="preserve">Priory Mews Care Home</t>
   </si>
   <si>
@@ -302,6 +326,9 @@
     <t xml:space="preserve">Independent nursing home in Dartford</t>
   </si>
   <si>
+    <t xml:space="preserve">Dr Marlon Zacarias Soriano (Registered Manager)</t>
+  </si>
+  <si>
     <t xml:space="preserve">St Aubyns Nursing Home</t>
   </si>
   <si>
@@ -323,6 +350,9 @@
     <t xml:space="preserve">Independent nursing home in Sidcup</t>
   </si>
   <si>
+    <t xml:space="preserve">Mrs Sheena John (Registered Manager)</t>
+  </si>
+  <si>
     <t xml:space="preserve">Antokol</t>
   </si>
   <si>
@@ -344,6 +374,9 @@
     <t xml:space="preserve">Nursing home in Chislehurst run by a charity</t>
   </si>
   <si>
+    <t xml:space="preserve">Mrs Joanna Wojtach (Registered Manager)</t>
+  </si>
+  <si>
     <t xml:space="preserve">Fairlight</t>
   </si>
   <si>
@@ -368,6 +401,9 @@
     <t xml:space="preserve">Mills Care Group: two homes in Chislehurst (Fairlight and Fallowfield)</t>
   </si>
   <si>
+    <t xml:space="preserve">Miss Tanya Angena Young (Registered Manager)</t>
+  </si>
+  <si>
     <t xml:space="preserve">Maples Care Home</t>
   </si>
   <si>
@@ -386,7 +422,10 @@
     <t xml:space="preserve">https://www.cqc.org.uk/location/1-21533595136</t>
   </si>
   <si>
-    <t xml:space="preserve">Independent nursing home in Bexleyheath</t>
+    <t xml:space="preserve">Independent nursing home in Bexleyheath. No Registered Manager listed on CQC: lead with manager recruitment</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Mr Antonio Kamal Carthigeya Thirulinganathan (Nominated Individual)</t>
   </si>
   <si>
     <t xml:space="preserve">Loring Hall Limited</t>
@@ -410,6 +449,9 @@
     <t xml:space="preserve">Learning disability residential service in Sidcup</t>
   </si>
   <si>
+    <t xml:space="preserve">Mr Paul Edward George Emile (Registered Manager)</t>
+  </si>
+  <si>
     <t xml:space="preserve">The Drive</t>
   </si>
   <si>
@@ -431,6 +473,9 @@
     <t xml:space="preserve">Small group of homes in Sidcup</t>
   </si>
   <si>
+    <t xml:space="preserve">Miss Abiola Oluwayemisi Odukale (Registered Manager)</t>
+  </si>
+  <si>
     <t xml:space="preserve">Groveland Park Care Home</t>
   </si>
   <si>
@@ -449,6 +494,9 @@
     <t xml:space="preserve">Independent residential home in Bexleyheath</t>
   </si>
   <si>
+    <t xml:space="preserve">Ms Caroline Susan Cheeseman (Registered Manager)</t>
+  </si>
+  <si>
     <t xml:space="preserve">Russell Court Nursing Home</t>
   </si>
   <si>
@@ -470,6 +518,9 @@
     <t xml:space="preserve">Independent nursing home near Longfield</t>
   </si>
   <si>
+    <t xml:space="preserve">Mrs Rachel Emma Caveney (Registered Manager)</t>
+  </si>
+  <si>
     <t xml:space="preserve">Bramblings Residential Home</t>
   </si>
   <si>
@@ -497,6 +548,9 @@
     <t xml:space="preserve">Independent residential home near Longfield</t>
   </si>
   <si>
+    <t xml:space="preserve">Mrs Jennifer Bard (Registered Manager)</t>
+  </si>
+  <si>
     <t xml:space="preserve">C</t>
   </si>
   <si>
@@ -524,6 +578,9 @@
     <t xml:space="preserve">Established Dartford home care provider</t>
   </si>
   <si>
+    <t xml:space="preserve">Mrs Jane Lisa Stevenson (Registered Manager)</t>
+  </si>
+  <si>
     <t xml:space="preserve">Athlone Care</t>
   </si>
   <si>
@@ -540,6 +597,9 @@
   </si>
   <si>
     <t xml:space="preserve">https://www.cqc.org.uk/location/1-437637829</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Mr David Mugwangi (Nominated Individual)</t>
   </si>
   <si>
     <t xml:space="preserve">Weekly targets</t>
@@ -1188,7 +1248,7 @@
     <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="16" min="16" style="0" width="20"/>
     <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="17" min="17" style="0" width="14"/>
     <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="18" min="18" style="0" width="12"/>
-    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="19" min="19" style="0" width="20"/>
+    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="19" min="19" style="0" width="36"/>
     <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="20" min="20" style="0" width="30"/>
   </cols>
   <sheetData>
@@ -1314,7 +1374,9 @@
         <f aca="false">IF(Q5="","",Q5+7)</f>
         <v/>
       </c>
-      <c r="S5" s="11"/>
+      <c r="S5" s="11" t="s">
+        <v>32</v>
+      </c>
       <c r="T5" s="11"/>
     </row>
     <row r="6" customFormat="false" ht="26.85" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -1328,37 +1390,37 @@
         <v>46293</v>
       </c>
       <c r="D6" s="7" t="s">
-        <v>32</v>
+        <v>33</v>
       </c>
       <c r="E6" s="8" t="s">
-        <v>33</v>
+        <v>34</v>
       </c>
       <c r="F6" s="9" t="s">
         <v>24</v>
       </c>
       <c r="G6" s="9" t="s">
-        <v>34</v>
+        <v>35</v>
       </c>
       <c r="H6" s="9" t="s">
-        <v>35</v>
+        <v>36</v>
       </c>
       <c r="I6" s="9" t="n">
         <v>2.9</v>
       </c>
       <c r="J6" s="9" t="s">
-        <v>36</v>
+        <v>37</v>
       </c>
       <c r="K6" s="9" t="s">
         <v>28</v>
       </c>
       <c r="L6" s="9" t="s">
-        <v>37</v>
+        <v>38</v>
       </c>
       <c r="M6" s="10" t="s">
-        <v>38</v>
+        <v>39</v>
       </c>
       <c r="N6" s="8" t="s">
-        <v>39</v>
+        <v>40</v>
       </c>
       <c r="O6" s="11"/>
       <c r="P6" s="11"/>
@@ -1367,7 +1429,9 @@
         <f aca="false">IF(Q6="","",Q6+7)</f>
         <v/>
       </c>
-      <c r="S6" s="11"/>
+      <c r="S6" s="11" t="s">
+        <v>41</v>
+      </c>
       <c r="T6" s="11"/>
     </row>
     <row r="7" customFormat="false" ht="26.85" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -1381,35 +1445,35 @@
         <v>46293</v>
       </c>
       <c r="D7" s="7" t="s">
-        <v>40</v>
+        <v>42</v>
       </c>
       <c r="E7" s="8" t="s">
-        <v>41</v>
+        <v>43</v>
       </c>
       <c r="F7" s="9" t="s">
         <v>24</v>
       </c>
       <c r="G7" s="9" t="s">
-        <v>42</v>
+        <v>44</v>
       </c>
       <c r="H7" s="9" t="s">
-        <v>43</v>
+        <v>45</v>
       </c>
       <c r="I7" s="9" t="n">
         <v>0.3</v>
       </c>
       <c r="J7" s="9" t="s">
-        <v>44</v>
+        <v>46</v>
       </c>
       <c r="K7" s="9" t="s">
         <v>28</v>
       </c>
       <c r="L7" s="9"/>
       <c r="M7" s="10" t="s">
-        <v>45</v>
+        <v>47</v>
       </c>
       <c r="N7" s="8" t="s">
-        <v>46</v>
+        <v>48</v>
       </c>
       <c r="O7" s="11"/>
       <c r="P7" s="11"/>
@@ -1418,7 +1482,9 @@
         <f aca="false">IF(Q7="","",Q7+7)</f>
         <v/>
       </c>
-      <c r="S7" s="11"/>
+      <c r="S7" s="11" t="s">
+        <v>49</v>
+      </c>
       <c r="T7" s="11"/>
     </row>
     <row r="8" customFormat="false" ht="26.85" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -1432,37 +1498,37 @@
         <v>46293</v>
       </c>
       <c r="D8" s="7" t="s">
-        <v>47</v>
+        <v>50</v>
       </c>
       <c r="E8" s="8" t="s">
-        <v>48</v>
+        <v>51</v>
       </c>
       <c r="F8" s="9" t="s">
-        <v>49</v>
+        <v>52</v>
       </c>
       <c r="G8" s="9" t="s">
-        <v>50</v>
+        <v>53</v>
       </c>
       <c r="H8" s="9" t="s">
-        <v>51</v>
+        <v>54</v>
       </c>
       <c r="I8" s="9" t="n">
         <v>6.3</v>
       </c>
       <c r="J8" s="9" t="s">
-        <v>52</v>
+        <v>55</v>
       </c>
       <c r="K8" s="9" t="s">
         <v>28</v>
       </c>
       <c r="L8" s="9" t="s">
-        <v>53</v>
+        <v>56</v>
       </c>
       <c r="M8" s="10" t="s">
-        <v>54</v>
+        <v>57</v>
       </c>
       <c r="N8" s="8" t="s">
-        <v>55</v>
+        <v>58</v>
       </c>
       <c r="O8" s="11"/>
       <c r="P8" s="11"/>
@@ -1471,7 +1537,9 @@
         <f aca="false">IF(Q8="","",Q8+7)</f>
         <v/>
       </c>
-      <c r="S8" s="11"/>
+      <c r="S8" s="11" t="s">
+        <v>59</v>
+      </c>
       <c r="T8" s="11"/>
     </row>
     <row r="9" customFormat="false" ht="26.85" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -1485,35 +1553,35 @@
         <v>46293</v>
       </c>
       <c r="D9" s="7" t="s">
-        <v>56</v>
+        <v>60</v>
       </c>
       <c r="E9" s="8" t="s">
-        <v>57</v>
+        <v>61</v>
       </c>
       <c r="F9" s="9" t="s">
         <v>24</v>
       </c>
       <c r="G9" s="9" t="s">
-        <v>58</v>
+        <v>62</v>
       </c>
       <c r="H9" s="9" t="s">
-        <v>59</v>
+        <v>63</v>
       </c>
       <c r="I9" s="9" t="n">
         <v>6.2</v>
       </c>
       <c r="J9" s="9" t="s">
-        <v>60</v>
+        <v>64</v>
       </c>
       <c r="K9" s="9" t="s">
         <v>28</v>
       </c>
       <c r="L9" s="9"/>
       <c r="M9" s="10" t="s">
-        <v>61</v>
+        <v>65</v>
       </c>
       <c r="N9" s="8" t="s">
-        <v>62</v>
+        <v>66</v>
       </c>
       <c r="O9" s="11"/>
       <c r="P9" s="11"/>
@@ -1522,7 +1590,9 @@
         <f aca="false">IF(Q9="","",Q9+7)</f>
         <v/>
       </c>
-      <c r="S9" s="11"/>
+      <c r="S9" s="11" t="s">
+        <v>67</v>
+      </c>
       <c r="T9" s="11"/>
     </row>
     <row r="10" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -1530,41 +1600,41 @@
         <v>6</v>
       </c>
       <c r="B10" s="9" t="s">
-        <v>63</v>
+        <v>68</v>
       </c>
       <c r="C10" s="6" t="n">
         <v>46294</v>
       </c>
       <c r="D10" s="8" t="s">
-        <v>64</v>
+        <v>69</v>
       </c>
       <c r="E10" s="8" t="s">
-        <v>65</v>
+        <v>70</v>
       </c>
       <c r="F10" s="9" t="s">
-        <v>66</v>
+        <v>71</v>
       </c>
       <c r="G10" s="9" t="s">
-        <v>42</v>
+        <v>44</v>
       </c>
       <c r="H10" s="9" t="s">
-        <v>67</v>
+        <v>72</v>
       </c>
       <c r="I10" s="9" t="n">
         <v>1.2</v>
       </c>
       <c r="J10" s="9" t="s">
-        <v>68</v>
+        <v>73</v>
       </c>
       <c r="K10" s="9" t="s">
         <v>28</v>
       </c>
       <c r="L10" s="9"/>
       <c r="M10" s="10" t="s">
-        <v>69</v>
+        <v>74</v>
       </c>
       <c r="N10" s="8" t="s">
-        <v>70</v>
+        <v>75</v>
       </c>
       <c r="O10" s="11"/>
       <c r="P10" s="11"/>
@@ -1573,7 +1643,9 @@
         <f aca="false">IF(Q10="","",Q10+7)</f>
         <v/>
       </c>
-      <c r="S10" s="11"/>
+      <c r="S10" s="11" t="s">
+        <v>76</v>
+      </c>
       <c r="T10" s="11"/>
     </row>
     <row r="11" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -1581,41 +1653,41 @@
         <v>7</v>
       </c>
       <c r="B11" s="9" t="s">
-        <v>63</v>
+        <v>68</v>
       </c>
       <c r="C11" s="6" t="n">
         <v>46294</v>
       </c>
       <c r="D11" s="8" t="s">
+        <v>77</v>
+      </c>
+      <c r="E11" s="8" t="s">
+        <v>78</v>
+      </c>
+      <c r="F11" s="9" t="s">
         <v>71</v>
       </c>
-      <c r="E11" s="8" t="s">
-        <v>72</v>
-      </c>
-      <c r="F11" s="9" t="s">
-        <v>66</v>
-      </c>
       <c r="G11" s="9" t="s">
-        <v>73</v>
+        <v>79</v>
       </c>
       <c r="H11" s="9" t="s">
-        <v>74</v>
+        <v>80</v>
       </c>
       <c r="I11" s="9" t="n">
         <v>3.4</v>
       </c>
       <c r="J11" s="9" t="s">
-        <v>75</v>
+        <v>81</v>
       </c>
       <c r="K11" s="9" t="s">
         <v>28</v>
       </c>
       <c r="L11" s="9"/>
       <c r="M11" s="10" t="s">
-        <v>76</v>
+        <v>82</v>
       </c>
       <c r="N11" s="8" t="s">
-        <v>77</v>
+        <v>83</v>
       </c>
       <c r="O11" s="11"/>
       <c r="P11" s="11"/>
@@ -1624,7 +1696,9 @@
         <f aca="false">IF(Q11="","",Q11+7)</f>
         <v/>
       </c>
-      <c r="S11" s="11"/>
+      <c r="S11" s="11" t="s">
+        <v>84</v>
+      </c>
       <c r="T11" s="11"/>
     </row>
     <row r="12" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -1632,43 +1706,43 @@
         <v>8</v>
       </c>
       <c r="B12" s="9" t="s">
-        <v>63</v>
+        <v>68</v>
       </c>
       <c r="C12" s="6" t="n">
         <v>46294</v>
       </c>
       <c r="D12" s="8" t="s">
-        <v>78</v>
+        <v>85</v>
       </c>
       <c r="E12" s="8" t="s">
+        <v>86</v>
+      </c>
+      <c r="F12" s="9" t="s">
+        <v>71</v>
+      </c>
+      <c r="G12" s="9" t="s">
         <v>79</v>
       </c>
-      <c r="F12" s="9" t="s">
-        <v>66</v>
-      </c>
-      <c r="G12" s="9" t="s">
-        <v>73</v>
-      </c>
       <c r="H12" s="9" t="s">
-        <v>80</v>
+        <v>87</v>
       </c>
       <c r="I12" s="9" t="n">
         <v>3.8</v>
       </c>
       <c r="J12" s="9" t="s">
-        <v>81</v>
+        <v>88</v>
       </c>
       <c r="K12" s="9" t="s">
-        <v>82</v>
+        <v>89</v>
       </c>
       <c r="L12" s="9" t="s">
-        <v>83</v>
+        <v>90</v>
       </c>
       <c r="M12" s="10" t="s">
-        <v>84</v>
+        <v>91</v>
       </c>
       <c r="N12" s="8" t="s">
-        <v>85</v>
+        <v>92</v>
       </c>
       <c r="O12" s="11"/>
       <c r="P12" s="11"/>
@@ -1677,7 +1751,9 @@
         <f aca="false">IF(Q12="","",Q12+7)</f>
         <v/>
       </c>
-      <c r="S12" s="11"/>
+      <c r="S12" s="11" t="s">
+        <v>93</v>
+      </c>
       <c r="T12" s="11"/>
     </row>
     <row r="13" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -1685,41 +1761,41 @@
         <v>9</v>
       </c>
       <c r="B13" s="9" t="s">
-        <v>63</v>
+        <v>68</v>
       </c>
       <c r="C13" s="6" t="n">
         <v>46294</v>
       </c>
       <c r="D13" s="8" t="s">
-        <v>86</v>
+        <v>94</v>
       </c>
       <c r="E13" s="8" t="s">
-        <v>87</v>
+        <v>95</v>
       </c>
       <c r="F13" s="9" t="s">
-        <v>66</v>
+        <v>71</v>
       </c>
       <c r="G13" s="9" t="s">
-        <v>73</v>
+        <v>79</v>
       </c>
       <c r="H13" s="9" t="s">
-        <v>88</v>
+        <v>96</v>
       </c>
       <c r="I13" s="9" t="n">
         <v>4.3</v>
       </c>
       <c r="J13" s="9" t="s">
-        <v>89</v>
+        <v>97</v>
       </c>
       <c r="K13" s="9" t="s">
         <v>28</v>
       </c>
       <c r="L13" s="9"/>
       <c r="M13" s="10" t="s">
-        <v>90</v>
+        <v>98</v>
       </c>
       <c r="N13" s="8" t="s">
-        <v>91</v>
+        <v>99</v>
       </c>
       <c r="O13" s="11"/>
       <c r="P13" s="11"/>
@@ -1728,7 +1804,9 @@
         <f aca="false">IF(Q13="","",Q13+7)</f>
         <v/>
       </c>
-      <c r="S13" s="11"/>
+      <c r="S13" s="11" t="s">
+        <v>100</v>
+      </c>
       <c r="T13" s="11"/>
     </row>
     <row r="14" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -1736,41 +1814,41 @@
         <v>10</v>
       </c>
       <c r="B14" s="9" t="s">
-        <v>63</v>
+        <v>68</v>
       </c>
       <c r="C14" s="6" t="n">
         <v>46294</v>
       </c>
       <c r="D14" s="8" t="s">
-        <v>92</v>
+        <v>101</v>
       </c>
       <c r="E14" s="8" t="s">
-        <v>93</v>
+        <v>102</v>
       </c>
       <c r="F14" s="9" t="s">
-        <v>66</v>
+        <v>71</v>
       </c>
       <c r="G14" s="9" t="s">
-        <v>94</v>
+        <v>103</v>
       </c>
       <c r="H14" s="9" t="s">
-        <v>95</v>
+        <v>104</v>
       </c>
       <c r="I14" s="9" t="n">
         <v>4.1</v>
       </c>
       <c r="J14" s="9" t="s">
-        <v>96</v>
+        <v>105</v>
       </c>
       <c r="K14" s="9" t="s">
         <v>28</v>
       </c>
       <c r="L14" s="9"/>
       <c r="M14" s="10" t="s">
-        <v>97</v>
+        <v>106</v>
       </c>
       <c r="N14" s="8" t="s">
-        <v>98</v>
+        <v>107</v>
       </c>
       <c r="O14" s="11"/>
       <c r="P14" s="11"/>
@@ -1779,7 +1857,9 @@
         <f aca="false">IF(Q14="","",Q14+7)</f>
         <v/>
       </c>
-      <c r="S14" s="11"/>
+      <c r="S14" s="11" t="s">
+        <v>108</v>
+      </c>
       <c r="T14" s="11"/>
     </row>
     <row r="15" customFormat="false" ht="26.85" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -1787,41 +1867,41 @@
         <v>11</v>
       </c>
       <c r="B15" s="9" t="s">
-        <v>63</v>
+        <v>68</v>
       </c>
       <c r="C15" s="6" t="n">
         <v>46294</v>
       </c>
       <c r="D15" s="8" t="s">
-        <v>99</v>
+        <v>109</v>
       </c>
       <c r="E15" s="8" t="s">
-        <v>100</v>
+        <v>110</v>
       </c>
       <c r="F15" s="9" t="s">
-        <v>66</v>
+        <v>71</v>
       </c>
       <c r="G15" s="9" t="s">
-        <v>101</v>
+        <v>111</v>
       </c>
       <c r="H15" s="9" t="s">
-        <v>102</v>
+        <v>112</v>
       </c>
       <c r="I15" s="9" t="n">
         <v>4.1</v>
       </c>
       <c r="J15" s="9" t="s">
-        <v>103</v>
+        <v>113</v>
       </c>
       <c r="K15" s="9" t="s">
         <v>28</v>
       </c>
       <c r="L15" s="9"/>
       <c r="M15" s="10" t="s">
-        <v>104</v>
+        <v>114</v>
       </c>
       <c r="N15" s="8" t="s">
-        <v>105</v>
+        <v>115</v>
       </c>
       <c r="O15" s="11"/>
       <c r="P15" s="11"/>
@@ -1830,7 +1910,9 @@
         <f aca="false">IF(Q15="","",Q15+7)</f>
         <v/>
       </c>
-      <c r="S15" s="11"/>
+      <c r="S15" s="11" t="s">
+        <v>116</v>
+      </c>
       <c r="T15" s="11"/>
     </row>
     <row r="16" customFormat="false" ht="26.85" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -1838,43 +1920,43 @@
         <v>12</v>
       </c>
       <c r="B16" s="9" t="s">
-        <v>63</v>
+        <v>68</v>
       </c>
       <c r="C16" s="6" t="n">
         <v>46294</v>
       </c>
       <c r="D16" s="8" t="s">
-        <v>106</v>
+        <v>117</v>
       </c>
       <c r="E16" s="8" t="s">
-        <v>107</v>
+        <v>118</v>
       </c>
       <c r="F16" s="9" t="s">
-        <v>108</v>
+        <v>119</v>
       </c>
       <c r="G16" s="9" t="s">
-        <v>101</v>
+        <v>111</v>
       </c>
       <c r="H16" s="9" t="s">
-        <v>109</v>
+        <v>120</v>
       </c>
       <c r="I16" s="9" t="n">
         <v>4.3</v>
       </c>
       <c r="J16" s="9" t="s">
-        <v>110</v>
+        <v>121</v>
       </c>
       <c r="K16" s="9" t="s">
         <v>28</v>
       </c>
       <c r="L16" s="9" t="s">
-        <v>111</v>
+        <v>122</v>
       </c>
       <c r="M16" s="10" t="s">
-        <v>112</v>
+        <v>123</v>
       </c>
       <c r="N16" s="8" t="s">
-        <v>113</v>
+        <v>124</v>
       </c>
       <c r="O16" s="11"/>
       <c r="P16" s="11"/>
@@ -1883,49 +1965,51 @@
         <f aca="false">IF(Q16="","",Q16+7)</f>
         <v/>
       </c>
-      <c r="S16" s="11"/>
+      <c r="S16" s="11" t="s">
+        <v>125</v>
+      </c>
       <c r="T16" s="11"/>
     </row>
-    <row r="17" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+    <row r="17" customFormat="false" ht="26.85" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A17" s="9" t="n">
         <v>13</v>
       </c>
       <c r="B17" s="9" t="s">
-        <v>63</v>
+        <v>68</v>
       </c>
       <c r="C17" s="6" t="n">
         <v>46295</v>
       </c>
       <c r="D17" s="8" t="s">
-        <v>114</v>
+        <v>126</v>
       </c>
       <c r="E17" s="8" t="s">
-        <v>115</v>
+        <v>127</v>
       </c>
       <c r="F17" s="9" t="s">
-        <v>66</v>
+        <v>71</v>
       </c>
       <c r="G17" s="9" t="s">
-        <v>116</v>
+        <v>128</v>
       </c>
       <c r="H17" s="9" t="s">
-        <v>117</v>
+        <v>129</v>
       </c>
       <c r="I17" s="9" t="n">
         <v>4.9</v>
       </c>
       <c r="J17" s="9" t="s">
-        <v>118</v>
+        <v>130</v>
       </c>
       <c r="K17" s="9" t="s">
         <v>28</v>
       </c>
       <c r="L17" s="9"/>
       <c r="M17" s="10" t="s">
-        <v>119</v>
+        <v>131</v>
       </c>
       <c r="N17" s="8" t="s">
-        <v>120</v>
+        <v>132</v>
       </c>
       <c r="O17" s="11"/>
       <c r="P17" s="11"/>
@@ -1934,7 +2018,9 @@
         <f aca="false">IF(Q17="","",Q17+7)</f>
         <v/>
       </c>
-      <c r="S17" s="11"/>
+      <c r="S17" s="11" t="s">
+        <v>133</v>
+      </c>
       <c r="T17" s="11"/>
     </row>
     <row r="18" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -1942,43 +2028,43 @@
         <v>14</v>
       </c>
       <c r="B18" s="9" t="s">
-        <v>63</v>
+        <v>68</v>
       </c>
       <c r="C18" s="6" t="n">
         <v>46295</v>
       </c>
       <c r="D18" s="8" t="s">
-        <v>121</v>
+        <v>134</v>
       </c>
       <c r="E18" s="8" t="s">
-        <v>122</v>
+        <v>135</v>
       </c>
       <c r="F18" s="9" t="s">
-        <v>108</v>
+        <v>119</v>
       </c>
       <c r="G18" s="9" t="s">
-        <v>94</v>
+        <v>103</v>
       </c>
       <c r="H18" s="9" t="s">
-        <v>123</v>
+        <v>136</v>
       </c>
       <c r="I18" s="9" t="n">
         <v>2.9</v>
       </c>
       <c r="J18" s="9" t="s">
-        <v>124</v>
+        <v>137</v>
       </c>
       <c r="K18" s="9" t="s">
         <v>28</v>
       </c>
       <c r="L18" s="9" t="s">
-        <v>125</v>
+        <v>138</v>
       </c>
       <c r="M18" s="10" t="s">
-        <v>126</v>
+        <v>139</v>
       </c>
       <c r="N18" s="8" t="s">
-        <v>127</v>
+        <v>140</v>
       </c>
       <c r="O18" s="11"/>
       <c r="P18" s="11"/>
@@ -1987,7 +2073,9 @@
         <f aca="false">IF(Q18="","",Q18+7)</f>
         <v/>
       </c>
-      <c r="S18" s="11"/>
+      <c r="S18" s="11" t="s">
+        <v>141</v>
+      </c>
       <c r="T18" s="11"/>
     </row>
     <row r="19" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -1995,43 +2083,43 @@
         <v>15</v>
       </c>
       <c r="B19" s="9" t="s">
-        <v>63</v>
+        <v>68</v>
       </c>
       <c r="C19" s="6" t="n">
         <v>46295</v>
       </c>
       <c r="D19" s="8" t="s">
-        <v>128</v>
+        <v>142</v>
       </c>
       <c r="E19" s="8" t="s">
-        <v>129</v>
+        <v>143</v>
       </c>
       <c r="F19" s="9" t="s">
-        <v>108</v>
+        <v>119</v>
       </c>
       <c r="G19" s="9" t="s">
-        <v>94</v>
+        <v>103</v>
       </c>
       <c r="H19" s="9" t="s">
-        <v>130</v>
+        <v>144</v>
       </c>
       <c r="I19" s="9" t="n">
         <v>3.4</v>
       </c>
       <c r="J19" s="9" t="s">
-        <v>131</v>
+        <v>145</v>
       </c>
       <c r="K19" s="9" t="s">
         <v>28</v>
       </c>
       <c r="L19" s="9" t="s">
-        <v>132</v>
+        <v>146</v>
       </c>
       <c r="M19" s="10" t="s">
-        <v>133</v>
+        <v>147</v>
       </c>
       <c r="N19" s="8" t="s">
-        <v>134</v>
+        <v>148</v>
       </c>
       <c r="O19" s="11"/>
       <c r="P19" s="11"/>
@@ -2040,7 +2128,9 @@
         <f aca="false">IF(Q19="","",Q19+7)</f>
         <v/>
       </c>
-      <c r="S19" s="11"/>
+      <c r="S19" s="11" t="s">
+        <v>149</v>
+      </c>
       <c r="T19" s="11"/>
     </row>
     <row r="20" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -2048,41 +2138,41 @@
         <v>16</v>
       </c>
       <c r="B20" s="9" t="s">
-        <v>63</v>
+        <v>68</v>
       </c>
       <c r="C20" s="6" t="n">
         <v>46295</v>
       </c>
       <c r="D20" s="8" t="s">
-        <v>135</v>
+        <v>150</v>
       </c>
       <c r="E20" s="8" t="s">
-        <v>136</v>
+        <v>151</v>
       </c>
       <c r="F20" s="9" t="s">
-        <v>108</v>
+        <v>119</v>
       </c>
       <c r="G20" s="9" t="s">
-        <v>116</v>
+        <v>128</v>
       </c>
       <c r="H20" s="9" t="s">
-        <v>137</v>
+        <v>152</v>
       </c>
       <c r="I20" s="9" t="n">
         <v>4.4</v>
       </c>
       <c r="J20" s="9" t="s">
-        <v>138</v>
+        <v>153</v>
       </c>
       <c r="K20" s="9" t="s">
         <v>28</v>
       </c>
       <c r="L20" s="9"/>
       <c r="M20" s="10" t="s">
-        <v>139</v>
+        <v>154</v>
       </c>
       <c r="N20" s="8" t="s">
-        <v>140</v>
+        <v>155</v>
       </c>
       <c r="O20" s="11"/>
       <c r="P20" s="11"/>
@@ -2091,7 +2181,9 @@
         <f aca="false">IF(Q20="","",Q20+7)</f>
         <v/>
       </c>
-      <c r="S20" s="11"/>
+      <c r="S20" s="11" t="s">
+        <v>156</v>
+      </c>
       <c r="T20" s="11"/>
     </row>
     <row r="21" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -2099,41 +2191,41 @@
         <v>17</v>
       </c>
       <c r="B21" s="9" t="s">
-        <v>63</v>
+        <v>68</v>
       </c>
       <c r="C21" s="6" t="n">
         <v>46295</v>
       </c>
       <c r="D21" s="8" t="s">
-        <v>141</v>
+        <v>157</v>
       </c>
       <c r="E21" s="8" t="s">
-        <v>142</v>
+        <v>158</v>
       </c>
       <c r="F21" s="9" t="s">
-        <v>66</v>
+        <v>71</v>
       </c>
       <c r="G21" s="9" t="s">
-        <v>143</v>
+        <v>159</v>
       </c>
       <c r="H21" s="9" t="s">
-        <v>144</v>
+        <v>160</v>
       </c>
       <c r="I21" s="9" t="n">
         <v>5.3</v>
       </c>
       <c r="J21" s="9" t="s">
-        <v>145</v>
+        <v>161</v>
       </c>
       <c r="K21" s="9" t="s">
         <v>28</v>
       </c>
       <c r="L21" s="9"/>
       <c r="M21" s="10" t="s">
-        <v>146</v>
+        <v>162</v>
       </c>
       <c r="N21" s="8" t="s">
-        <v>147</v>
+        <v>163</v>
       </c>
       <c r="O21" s="11"/>
       <c r="P21" s="11"/>
@@ -2142,7 +2234,9 @@
         <f aca="false">IF(Q21="","",Q21+7)</f>
         <v/>
       </c>
-      <c r="S21" s="11"/>
+      <c r="S21" s="11" t="s">
+        <v>164</v>
+      </c>
       <c r="T21" s="11"/>
     </row>
     <row r="22" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -2150,43 +2244,43 @@
         <v>18</v>
       </c>
       <c r="B22" s="9" t="s">
-        <v>63</v>
+        <v>68</v>
       </c>
       <c r="C22" s="6" t="n">
         <v>46295</v>
       </c>
       <c r="D22" s="8" t="s">
-        <v>148</v>
+        <v>165</v>
       </c>
       <c r="E22" s="8" t="s">
-        <v>149</v>
+        <v>166</v>
       </c>
       <c r="F22" s="9" t="s">
-        <v>108</v>
+        <v>119</v>
       </c>
       <c r="G22" s="9" t="s">
-        <v>150</v>
+        <v>167</v>
       </c>
       <c r="H22" s="9" t="s">
-        <v>151</v>
+        <v>168</v>
       </c>
       <c r="I22" s="9" t="n">
         <v>5.5</v>
       </c>
       <c r="J22" s="9" t="s">
-        <v>152</v>
+        <v>169</v>
       </c>
       <c r="K22" s="9" t="s">
-        <v>153</v>
+        <v>170</v>
       </c>
       <c r="L22" s="9" t="s">
-        <v>154</v>
+        <v>171</v>
       </c>
       <c r="M22" s="10" t="s">
-        <v>155</v>
+        <v>172</v>
       </c>
       <c r="N22" s="8" t="s">
-        <v>156</v>
+        <v>173</v>
       </c>
       <c r="O22" s="11"/>
       <c r="P22" s="11"/>
@@ -2195,7 +2289,9 @@
         <f aca="false">IF(Q22="","",Q22+7)</f>
         <v/>
       </c>
-      <c r="S22" s="11"/>
+      <c r="S22" s="11" t="s">
+        <v>174</v>
+      </c>
       <c r="T22" s="11"/>
     </row>
     <row r="23" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -2203,43 +2299,43 @@
         <v>19</v>
       </c>
       <c r="B23" s="9" t="s">
-        <v>157</v>
+        <v>175</v>
       </c>
       <c r="C23" s="6" t="n">
         <v>46295</v>
       </c>
       <c r="D23" s="8" t="s">
-        <v>158</v>
+        <v>176</v>
       </c>
       <c r="E23" s="8" t="s">
-        <v>159</v>
+        <v>177</v>
       </c>
       <c r="F23" s="9" t="s">
         <v>24</v>
       </c>
       <c r="G23" s="9" t="s">
-        <v>73</v>
+        <v>79</v>
       </c>
       <c r="H23" s="9" t="s">
-        <v>160</v>
+        <v>178</v>
       </c>
       <c r="I23" s="9" t="n">
         <v>2.4</v>
       </c>
       <c r="J23" s="9" t="s">
-        <v>161</v>
+        <v>179</v>
       </c>
       <c r="K23" s="9" t="s">
-        <v>162</v>
+        <v>180</v>
       </c>
       <c r="L23" s="9" t="s">
-        <v>163</v>
+        <v>181</v>
       </c>
       <c r="M23" s="10" t="s">
-        <v>164</v>
+        <v>182</v>
       </c>
       <c r="N23" s="8" t="s">
-        <v>165</v>
+        <v>183</v>
       </c>
       <c r="O23" s="11"/>
       <c r="P23" s="11"/>
@@ -2248,7 +2344,9 @@
         <f aca="false">IF(Q23="","",Q23+7)</f>
         <v/>
       </c>
-      <c r="S23" s="11"/>
+      <c r="S23" s="11" t="s">
+        <v>184</v>
+      </c>
       <c r="T23" s="11"/>
     </row>
     <row r="24" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -2256,43 +2354,43 @@
         <v>20</v>
       </c>
       <c r="B24" s="9" t="s">
-        <v>157</v>
+        <v>175</v>
       </c>
       <c r="C24" s="6" t="n">
         <v>46295</v>
       </c>
       <c r="D24" s="8" t="s">
-        <v>166</v>
+        <v>185</v>
       </c>
       <c r="E24" s="8" t="s">
-        <v>167</v>
+        <v>186</v>
       </c>
       <c r="F24" s="9" t="s">
         <v>24</v>
       </c>
       <c r="G24" s="9" t="s">
-        <v>73</v>
+        <v>79</v>
       </c>
       <c r="H24" s="9" t="s">
-        <v>168</v>
+        <v>187</v>
       </c>
       <c r="I24" s="9" t="n">
         <v>3.9</v>
       </c>
       <c r="J24" s="9" t="s">
-        <v>169</v>
+        <v>188</v>
       </c>
       <c r="K24" s="9" t="s">
         <v>28</v>
       </c>
       <c r="L24" s="9" t="s">
-        <v>170</v>
+        <v>189</v>
       </c>
       <c r="M24" s="10" t="s">
-        <v>171</v>
+        <v>190</v>
       </c>
       <c r="N24" s="8" t="s">
-        <v>165</v>
+        <v>183</v>
       </c>
       <c r="O24" s="11"/>
       <c r="P24" s="11"/>
@@ -2301,28 +2399,30 @@
         <f aca="false">IF(Q24="","",Q24+7)</f>
         <v/>
       </c>
-      <c r="S24" s="11"/>
+      <c r="S24" s="11" t="s">
+        <v>191</v>
+      </c>
       <c r="T24" s="11"/>
     </row>
     <row r="26" customFormat="false" ht="16.15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A26" s="13" t="s">
-        <v>172</v>
+        <v>192</v>
       </c>
     </row>
     <row r="27" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="D27" s="14" t="s">
-        <v>173</v>
+        <v>193</v>
       </c>
       <c r="E27" s="14" t="s">
-        <v>174</v>
+        <v>194</v>
       </c>
       <c r="F27" s="14" t="s">
-        <v>175</v>
+        <v>195</v>
       </c>
     </row>
     <row r="28" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="D28" s="15" t="s">
-        <v>176</v>
+        <v>196</v>
       </c>
       <c r="E28" s="14" t="n">
         <f aca="false">COUNTA(P5:P24)</f>
@@ -2334,7 +2434,7 @@
     </row>
     <row r="29" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="D29" s="15" t="s">
-        <v>177</v>
+        <v>197</v>
       </c>
       <c r="E29" s="14" t="n">
         <f aca="false">COUNT(Q5:Q24)</f>
@@ -2346,7 +2446,7 @@
     </row>
     <row r="30" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="D30" s="15" t="s">
-        <v>178</v>
+        <v>198</v>
       </c>
       <c r="E30" s="14" t="n">
         <f aca="false">COUNTIF(P5:P24,"Meeting booked")</f>
@@ -2358,7 +2458,7 @@
     </row>
     <row r="31" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="D31" s="15" t="s">
-        <v>179</v>
+        <v>199</v>
       </c>
       <c r="E31" s="14" t="n">
         <f aca="false">COUNTIF(P5:P24,"Has a vacancy")</f>
@@ -2428,79 +2528,79 @@
   <sheetData>
     <row r="1" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A1" s="16" t="s">
-        <v>180</v>
+        <v>200</v>
       </c>
       <c r="B1" s="16" t="s">
-        <v>181</v>
+        <v>201</v>
       </c>
       <c r="C1" s="16" t="s">
-        <v>182</v>
+        <v>202</v>
       </c>
     </row>
     <row r="2" customFormat="false" ht="26.85" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A2" s="17" t="s">
-        <v>183</v>
+        <v>203</v>
       </c>
       <c r="B2" s="17" t="s">
-        <v>184</v>
+        <v>204</v>
       </c>
       <c r="C2" s="17" t="s">
-        <v>185</v>
+        <v>205</v>
       </c>
     </row>
     <row r="3" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A3" s="17" t="s">
-        <v>186</v>
+        <v>206</v>
       </c>
       <c r="B3" s="17" t="s">
-        <v>187</v>
+        <v>207</v>
       </c>
       <c r="C3" s="17" t="s">
-        <v>188</v>
+        <v>208</v>
       </c>
     </row>
     <row r="4" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A4" s="17" t="s">
-        <v>189</v>
+        <v>209</v>
       </c>
       <c r="B4" s="17" t="s">
-        <v>190</v>
+        <v>210</v>
       </c>
       <c r="C4" s="17" t="s">
-        <v>188</v>
+        <v>208</v>
       </c>
     </row>
     <row r="5" customFormat="false" ht="26.85" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A5" s="17" t="s">
-        <v>191</v>
+        <v>211</v>
       </c>
       <c r="B5" s="17" t="s">
-        <v>192</v>
+        <v>212</v>
       </c>
       <c r="C5" s="17" t="s">
-        <v>193</v>
+        <v>213</v>
       </c>
     </row>
     <row r="6" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A6" s="17" t="s">
-        <v>194</v>
+        <v>214</v>
       </c>
       <c r="B6" s="17" t="s">
-        <v>195</v>
+        <v>215</v>
       </c>
       <c r="C6" s="17" t="s">
-        <v>196</v>
+        <v>216</v>
       </c>
     </row>
     <row r="7" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A7" s="17" t="s">
-        <v>197</v>
+        <v>217</v>
       </c>
       <c r="B7" s="17" t="s">
-        <v>198</v>
+        <v>218</v>
       </c>
       <c r="C7" s="17" t="s">
-        <v>193</v>
+        <v>213</v>
       </c>
     </row>
   </sheetData>

</xml_diff>